<commit_message>
Fix Tajima's grade to Associate (A) and convert workbook font to Meiryo UI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TEpt4sX19FFE6MDm3ugNoG
</commit_message>
<xml_diff>
--- a/INTS_HRキャリアパス設計_既存情報整理とヒアリング項目_v01.xlsx
+++ b/INTS_HRキャリアパス設計_既存情報整理とヒアリング項目_v01.xlsx
@@ -32,35 +32,35 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Meiryo UI"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -790,7 +790,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>As-Is体制。HRラインはM・Cのみ</t>
+          <t>As-Is体制。HRラインはM・Aのみ</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Director 福島（Corp Planning 0.5FTE）の下にHRライン（小出：Manager − 田嶋：Consultant）とFINライン（東：SC − SC-A：採用予定）</t>
+          <t>Director 福島（Corp Planning 0.5FTE）の下にHRライン（小出：Manager − 田嶋：Associate）とFINライン（東：SC − SC-A：採用予定）</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>HRラインに今いるのはMとCのみ。A／SC／SM層とHR専任のDirector層は空席 → キャリアパスは「いない層の役割定義」が中心になる</t>
+          <t>HRラインに今いるのはMとAのみ。C／SC／SM層とHR専任のDirector層は空席 → キャリアパスは「いない層の役割定義」が中心になる</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>田嶋（A）</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>田嶋</t>
+          <t>-（空席）</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr"/>

</xml_diff>